<commit_message>
Convert to static site (Feb 2026)
</commit_message>
<xml_diff>
--- a/static/data/Extended-Indexes.xlsx
+++ b/static/data/Extended-Indexes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ441"/>
+  <dimension ref="A1:AQ442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51079,19 +51079,19 @@
         </is>
       </c>
       <c r="B441" t="n">
-        <v>16.66666666666666</v>
+        <v>15.38461538461539</v>
       </c>
       <c r="C441" t="n">
         <v>0</v>
       </c>
       <c r="D441" t="n">
-        <v>58.33333333333334</v>
+        <v>53.84615384615385</v>
       </c>
       <c r="E441" t="n">
-        <v>76.92307692307693</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="F441" t="n">
-        <v>16.66666666666666</v>
+        <v>15.38461538461539</v>
       </c>
       <c r="G441" t="n">
         <v>40916.41666666666</v>
@@ -51100,31 +51100,31 @@
         <v>-0.4444444444444444</v>
       </c>
       <c r="I441" t="n">
-        <v>-0.3750000000000001</v>
+        <v>-0.5769230769230771</v>
       </c>
       <c r="J441" t="n">
         <v>0</v>
       </c>
       <c r="K441" t="n">
-        <v>-0.8333333333333334</v>
+        <v>-0.3846153846153847</v>
       </c>
       <c r="L441" t="n">
         <v>3.888888888888889</v>
       </c>
       <c r="M441" t="n">
-        <v>-0.3749999999999998</v>
+        <v>0.0384615384615386</v>
       </c>
       <c r="N441" t="n">
         <v>6.909090909090909</v>
       </c>
       <c r="O441" t="n">
-        <v>3.772727272727272</v>
+        <v>1.791666666666667</v>
       </c>
       <c r="P441" t="n">
         <v>43.22727272727272</v>
       </c>
       <c r="Q441" t="n">
-        <v>56.89999999999999</v>
+        <v>52.63636363636364</v>
       </c>
       <c r="R441" t="n">
         <v>1.666666666666667</v>
@@ -51142,55 +51142,55 @@
         <v>36.25</v>
       </c>
       <c r="W441" t="n">
-        <v>33.33333333333333</v>
+        <v>30.76923076923077</v>
       </c>
       <c r="X441" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y441" t="n">
+        <v>7.692307692307693</v>
+      </c>
+      <c r="Z441" t="n">
+        <v>42.85714285714285</v>
+      </c>
+      <c r="AA441" t="n">
         <v>69.23076923076923</v>
       </c>
-      <c r="Y441" t="n">
-        <v>8.333333333333332</v>
-      </c>
-      <c r="Z441" t="n">
-        <v>41.66666666666667</v>
-      </c>
-      <c r="AA441" t="n">
-        <v>75</v>
-      </c>
       <c r="AB441" t="n">
-        <v>76.92307692307693</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="AC441" t="n">
-        <v>58.33333333333334</v>
+        <v>53.84615384615385</v>
       </c>
       <c r="AD441" t="n">
+        <v>46.66666666666666</v>
+      </c>
+      <c r="AE441" t="n">
+        <v>25.76923076923077</v>
+      </c>
+      <c r="AF441" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AG441" t="n">
         <v>46.15384615384615</v>
       </c>
-      <c r="AE441" t="n">
-        <v>23.75</v>
-      </c>
-      <c r="AF441" t="n">
-        <v>24.03846153846154</v>
-      </c>
-      <c r="AG441" t="n">
-        <v>41.66666666666667</v>
-      </c>
       <c r="AH441" t="n">
-        <v>76.92307692307693</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="AI441" t="n">
-        <v>66.66666666666666</v>
+        <v>61.53846153846154</v>
       </c>
       <c r="AJ441" t="n">
-        <v>84.61538461538461</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="AK441" t="n">
         <v>58.33333333333334</v>
       </c>
       <c r="AL441" t="n">
-        <v>30.76923076923077</v>
+        <v>26.66666666666667</v>
       </c>
       <c r="AM441" t="n">
-        <v>3.229166666666667</v>
+        <v>4.903846153846154</v>
       </c>
       <c r="AN441" t="n">
         <v>8.375</v>
@@ -51203,6 +51203,139 @@
       </c>
       <c r="AQ441" t="n">
         <v>17.06</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B442" t="n">
+        <v>0</v>
+      </c>
+      <c r="C442" t="n">
+        <v>0</v>
+      </c>
+      <c r="D442" t="n">
+        <v>41.66666666666667</v>
+      </c>
+      <c r="E442" t="n">
+        <v>56.52173913043478</v>
+      </c>
+      <c r="F442" t="n">
+        <v>9.090909090909092</v>
+      </c>
+      <c r="G442" t="n">
+        <v>48321.2</v>
+      </c>
+      <c r="H442" t="n">
+        <v>1.272727272727273</v>
+      </c>
+      <c r="I442" t="n">
+        <v>0.3760000000000001</v>
+      </c>
+      <c r="J442" t="n">
+        <v>0.6136363636363636</v>
+      </c>
+      <c r="K442" t="n">
+        <v>0.6755</v>
+      </c>
+      <c r="L442" t="n">
+        <v>1.590909090909091</v>
+      </c>
+      <c r="M442" t="n">
+        <v>-1.825</v>
+      </c>
+      <c r="N442" t="n">
+        <v>4.636363636363637</v>
+      </c>
+      <c r="O442" t="n">
+        <v>-0.9473684210526314</v>
+      </c>
+      <c r="P442" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q442" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="R442" t="n">
+        <v>1.571428571428572</v>
+      </c>
+      <c r="S442" t="n">
+        <v>5</v>
+      </c>
+      <c r="T442" t="n">
+        <v>6.857142857142858</v>
+      </c>
+      <c r="U442" t="n">
+        <v>7.142857142857142</v>
+      </c>
+      <c r="V442" t="n">
+        <v>50</v>
+      </c>
+      <c r="W442" t="n">
+        <v>54.54545454545454</v>
+      </c>
+      <c r="X442" t="n">
+        <v>43.47826086956522</v>
+      </c>
+      <c r="Y442" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z442" t="n">
+        <v>34.78260869565217</v>
+      </c>
+      <c r="AA442" t="n">
+        <v>58.33333333333334</v>
+      </c>
+      <c r="AB442" t="n">
+        <v>78.26086956521739</v>
+      </c>
+      <c r="AC442" t="n">
+        <v>75</v>
+      </c>
+      <c r="AD442" t="n">
+        <v>65.21739130434783</v>
+      </c>
+      <c r="AE442" t="n">
+        <v>11.16666666666667</v>
+      </c>
+      <c r="AF442" t="n">
+        <v>22.33181818181818</v>
+      </c>
+      <c r="AG442" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="AH442" t="n">
+        <v>69.56521739130434</v>
+      </c>
+      <c r="AI442" t="n">
+        <v>83.33333333333334</v>
+      </c>
+      <c r="AJ442" t="n">
+        <v>65.21739130434783</v>
+      </c>
+      <c r="AK442" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="AL442" t="n">
+        <v>43.47826086956522</v>
+      </c>
+      <c r="AM442" t="n">
+        <v>2.961666666666667</v>
+      </c>
+      <c r="AN442" t="n">
+        <v>10.31666666666667</v>
+      </c>
+      <c r="AO442" t="n">
+        <v>7.555555555555555</v>
+      </c>
+      <c r="AP442" t="n">
+        <v>8.191666666666668</v>
+      </c>
+      <c r="AQ442" t="n">
+        <v>6.466666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>